<commit_message>
Kopieen in Per visite byte-gelijk met Per nummer
Negen kopieen hadden dezelfde tekst (resp. dezelfde celwaarden) als de werkset,
maar waren apart opgeslagen: 09b in vijf visitemappen, 32 in V7 en V8, 45a in V1,
en de identificatielijst 00 in V0 (werkset van 4 augustus, visitekopie van 29
juli; alle zeven bladen dezelfde waarden). Nu byte-identiek.

Na deze stap zijn alle 141 kopieen in Per visite identiek aan Per nummer. De 47
documenten in Per protocolnaam verschillen alleen in de titelregel (eCRF Document
NN: protocolnaam), zoals die map bedoeld is.

eCRF 21 (Vlaamse EQ-5D-5L) is lokaal in alle negen mappen bijgewerkt maar bewust
niet gecommit: de repo is openbaar en EuroQol staat niet toe dat het instrument
openbaar gemaakt wordt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/(e)CRF/Per visite/V0 - Screening/00_Patienten-identificatielijst.xlsx
+++ b/(e)CRF/Per visite/V0 - Screening/00_Patienten-identificatielijst.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="152" documentId="8_{79E5BB8D-1D9C-4A86-B32A-DAD463DBE238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F4420E-4239-40F8-99A5-2E4EAD59267D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{BAE69EEB-DB30-489E-A1E1-995352FC35D1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BAE69EEB-DB30-489E-A1E1-995352FC35D1}"/>
   </bookViews>
   <sheets>
     <sheet name="UZ Leuven" sheetId="1" r:id="rId1"/>
@@ -14245,6 +14245,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F1B33D7B57FFEC4BB77B5001C5B93838" ma:contentTypeVersion="6" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="59579db12405a868ad0e92c5e4f74ae1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f44e6bd5-09db-4117-8b15-adf399208dc6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="98cf673e6ff17a9b7a889e3f7df574b2" ns2:_="">
     <xsd:import namespace="f44e6bd5-09db-4117-8b15-adf399208dc6"/>
@@ -14400,22 +14415,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BDCF903-BA31-4DB0-B467-C3CC1B28989E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88182F73-E0BA-40D2-A01B-FE2F1A72F50B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F72EF480-3E9C-466F-BA1A-D34CBC3C9DDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -14431,21 +14448,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88182F73-E0BA-40D2-A01B-FE2F1A72F50B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BDCF903-BA31-4DB0-B467-C3CC1B28989E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>